<commit_message>
Deploy TWHA IG: Wave 7 委員意見處置 (狀態標示/SNOMED隔離/subject修正/三層說明)
對應原始碼 commit 5b03d090。以 tx.fhir.org 驗證通過(語法與已被引用術語)。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CodeSystem-CS-Appendix10Operation.xlsx
+++ b/CodeSystem-CS-Appendix10Operation.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-26T12:18:37+08:00</t>
+    <t>2026-07-26T14:28:30+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>《勞工健康保護規則》附表十（115.06.26 修正）逐號列舉之 35 項特別危害健康作業具名代碼。本代碼系統為「具名作業層」，與 CS-HazardType（12 危害家族層）以 ConceptMap Appendix10-to-HazardType 對映。編號 33/34/35（苯乙烯、甲苯、二甲苯）為 115.06.26 修正新增。</t>
+    <t>《勞工健康保護規則》附表十（115.06.26 修正）逐號列舉之 35 項特別危害健康作業具名代碼。本代碼系統為「具名作業層」，與 CS-HazardType（12 危害家族層）以 ConceptMap Appendix10-to-HazardType 對映。編號 33/34/35（苯乙烯、甲苯、二甲苯）為 115.06.26 修正新增，狀態為 **draft**：其施行日期與既有勞工銜接安排尚待勞動部職業安全衛生署確認，本 IG 之檢查項目與代碼配置屬暫定。過渡期以本 CodeSystem 之 version（法規版本）表達，個案資料僅記錄實際檢查日期與所採規範版本，不另加自訂旗標。</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>